<commit_message>
fix: parse FSH files directement (fsh-generated ignoré par git)
- Le script lisait fsh-generated/resources/ qui est dans .gitignore
  et donc absent en CI → Excel vide
- Nouveau parseur FSH sur input/fsh/logicals/**/*.fsh
- Lien de téléchargement déplacé en bas de la page d'accueil

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/input/images/MOS.xlsx
+++ b/input/images/MOS.xlsx
@@ -1163,7 +1163,7 @@
       <c r="E25" s="3" t="n"/>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>Extrait du rapport de l'ONDPS sur la médecine générale (Tome 1 2006-2007): "La compétence était un titre délivré par l’ordre national des médecins en application du précédent règlement de qualification (Article 3 de l'arrêté du 4 septembre 1970), aux praticiens dits «ancien régime» ayant débuté leurs études médicales avant la réforme de 1982. Ce titre était accordé après avis d’une commission ordinale spécifique. Les compétences, dont la liste était fixée par arrêté, portaient soit sur des disciplines ne correspondant pas à des spécialités qualifiantes (médecine légale ou allergologie par exemple), soit sur des spécialités médicales, le praticien compétent ne pouvant l’exercer que dans le cadre de sa spécialité d’inscription à l’ordre. Les compétences ne peuvent plus être délivrées aux médecins issus du nouveau régime, c’est-à-dire ayant débuté leurs études à compter de l’année universitaire 1984-1985. Toutefois, pour ceux de l’ancien régime et à titre transitoire, le dépôt d’une demande de qualification était possible jusqu’au 31 décembre 2004 et ces praticiens peuvent s’en prévaloir jusqu’à la fin leur période d’activité professionnelle.Une compétence est un type de savoir-faire. La classe Competence est représentée dans le modèle comme une spécialisation de la classe SavoirFaire et à ce titre, elle hérite des attributs et des associations de cette classe.</t>
+          <t>Extrait du rapport de l'ONDPS sur la médecine générale (Tome 1 2006-2007): \"La compétence était un titre délivré par l’ordre national des médecins en application du précédent règlement de qualification (Article 3 de l'arrêté du 4 septembre 1970), aux praticiens dits «ancien régime» ayant débuté leurs études médicales avant la réforme de 1982. Ce titre était accordé après avis d’une commission ordinale spécifique. Les compétences, dont la liste était fixée par arrêté, portaient soit sur des disciplines ne correspondant pas à des spécialités qualifiantes (médecine légale ou allergologie par exemple), soit sur des spécialités médicales, le praticien compétent ne pouvant l’exercer que dans le cadre de sa spécialité d’inscription à l’ordre. Les compétences ne peuvent plus être délivrées aux médecins issus du nouveau régime, c’est-à-dire ayant débuté leurs études à compter de l’année universitaire 1984-1985. Toutefois, pour ceux de l’ancien régime et à titre transitoire, le dépôt d’une demande de qualification était possible jusqu’au 31 décembre 2004 et ces praticiens peuvent s’en prévaloir jusqu’à la fin leur période d’activité professionnelle.Une compétence est un type de savoir-faire. La classe Competence est représentée dans le modèle comme une spécialisation de la classe SavoirFaire et à ce titre, elle hérite des attributs et des associations de cette classe.</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr"/>
@@ -1337,7 +1337,7 @@
       <c r="E31" s="3" t="n"/>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>Expérience pratique exigée par le code de la santé publique (art R5124-16) pour exercer certaines fonctions dans l’industrie pharmaceutique et la distribution en gros. Ces dispositions s’appliquent uniquement à la profession de pharmacien.L’expérience pratique est en liaison avec les activités de l’établissement pharmaceutique telles que définies par l’ANSM ou l’ANSES.A ce jour, cinq expériences pratiques sont identifiées dont trois sont imbriquées. L’expérience pratique de "Fabricant" inclut celle d’"Exploitant" qui inclut celle de "Distribution".  Une fonction qualifiée est un type de savoir-faire. La classe FonctionQualifiee est représentée dans le modèle comme une spécialisation de la classe SavoirFaire et à ce titre, elle hérite des attributs et des associations de cette classe.</t>
+          <t>Expérience pratique exigée par le code de la santé publique (art R5124-16) pour exercer certaines fonctions dans l’industrie pharmaceutique et la distribution en gros. Ces dispositions s’appliquent uniquement à la profession de pharmacien.L’expérience pratique est en liaison avec les activités de l’établissement pharmaceutique telles que définies par l’ANSM ou l’ANSES.A ce jour, cinq expériences pratiques sont identifiées dont trois sont imbriquées. L’expérience pratique de \"Fabricant\" inclut celle d’\"Exploitant\" qui inclut celle de \"Distribution\".  Une fonction qualifiée est un type de savoir-faire. La classe FonctionQualifiee est représentée dans le modèle comme une spécialisation de la classe SavoirFaire et à ce titre, elle hérite des attributs et des associations de cette classe.</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr"/>
@@ -1859,7 +1859,7 @@
       <c r="E49" s="3" t="n"/>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>Loi HPST, art.13: "Pour les établissements publics de santé, le directeur définit l'organisation de l'établissement en pôles d'activité conformément au projet médical d'établissement, après avis [...]. Le directeur général de l'agence régionale de santé peut autoriser un établissement à ne pas créer de pôles d'activité quand l'effectif médical de l'établissement le justifie.Les pôles d'activité peuvent comporter des structures internes de prise en charge du malade par les équipes médicales, soignantes ou médico-techniques ainsi que les structures médico-techniques qui leur sont associées".Extrait de "La loi HPST à l'hôpital, les clés pour comprendre - Ministère de la Santé- ANAP": "Les pôles d’activité clinique et médico-technique peuvent comporter des "structures internes" de prise en charge du malade par les équipes médicales, soignantes ou médico-techniques".Les pôles peuvent être multi-sites, c'est à dire qu'un même pôle peut comporter des structures internes situées dans différentes entités géographiques d'une même entité juridique.</t>
+          <t>Loi HPST, art.13: \"Pour les établissements publics de santé, le directeur définit l'organisation de l'établissement en pôles d'activité conformément au projet médical d'établissement, après avis [...]. Le directeur général de l'agence régionale de santé peut autoriser un établissement à ne pas créer de pôles d'activité quand l'effectif médical de l'établissement le justifie.Les pôles d'activité peuvent comporter des structures internes de prise en charge du malade par les équipes médicales, soignantes ou médico-techniques ainsi que les structures médico-techniques qui leur sont associées\".Extrait de \"La loi HPST à l'hôpital, les clés pour comprendre - Ministère de la Santé- ANAP\": \"Les pôles d’activité clinique et médico-technique peuvent comporter des \"structures internes\" de prise en charge du malade par les équipes médicales, soignantes ou médico-techniques\".Les pôles peuvent être multi-sites, c'est à dire qu'un même pôle peut comporter des structures internes situées dans différentes entités géographiques d'une même entité juridique.</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr"/>
@@ -1888,7 +1888,7 @@
       <c r="E50" s="3" t="n"/>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>Une structure interne peut être composée d'une ou plusieurs unités médicales fonctionnelles.L’appellation des structures internes des pôles est aussi laissée à la libre appréciation des établissements : il peut s’agir de services, d’unités, de centres, d’instituts, de départements, ou de toute autre appellation. Lorsque les services demeurent, les chefs de service sont placés sous l’autorité fonctionnelle du chef de pôle (cf. "La loi HPST à l'hôpital, les clés pour comprendre" - Ministère de la Santé - ANAP).Synonyme : Service, unité, centre, institut, département, etc.</t>
+          <t>Une structure interne peut être composée d'une ou plusieurs unités médicales fonctionnelles.L’appellation des structures internes des pôles est aussi laissée à la libre appréciation des établissements : il peut s’agir de services, d’unités, de centres, d’instituts, de départements, ou de toute autre appellation. Lorsque les services demeurent, les chefs de service sont placés sous l’autorité fonctionnelle du chef de pôle (cf. \"La loi HPST à l'hôpital, les clés pour comprendre\" - Ministère de la Santé - ANAP).Synonyme : Service, unité, centre, institut, département, etc.</t>
         </is>
       </c>
       <c r="G50" s="3" t="inlineStr"/>
@@ -2091,7 +2091,7 @@
       <c r="E57" s="3" t="n"/>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>/!\ Classe en cours de constructionInformations relatives à la vie quotidienne de la personne prise en charge.</t>
+          <t>/!\\ Classe en cours de constructionInformations relatives à la vie quotidienne de la personne prise en charge.</t>
         </is>
       </c>
       <c r="G57" s="3" t="inlineStr"/>
@@ -2120,7 +2120,7 @@
       <c r="E58" s="3" t="n"/>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>/!\ Classe en cours de constructionInformations relatives à la vie professionnelle de la personne prise en charge.</t>
+          <t>/!\\ Classe en cours de constructionInformations relatives à la vie professionnelle de la personne prise en charge.</t>
         </is>
       </c>
       <c r="G58" s="3" t="inlineStr"/>
@@ -2207,7 +2207,7 @@
       <c r="E61" s="3" t="n"/>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>/!\ Classe en cours de constructionInformations relatives à la vie scolaire de la personne prise en charge.</t>
+          <t>/!\\ Classe en cours de constructionInformations relatives à la vie scolaire de la personne prise en charge.</t>
         </is>
       </c>
       <c r="G61" s="3" t="inlineStr"/>
@@ -3019,7 +3019,7 @@
       <c r="E89" s="3" t="n"/>
       <c r="F89" s="3" t="inlineStr">
         <is>
-          <t>Un diplôme sanctionne un niveau de connaissances. L’Etat intervient, dans certains cas, sur le programme et la pédagogie de certains cursus diplômants, par exemple les diplômes d'Etat.La classe "Diplome" est une classe générale contenant les propriétés communes aux différents types de diplômes.Chaque diplôme est décrit dans le modèle comme une spécialisation de la classe Diplome et à ce titre, hérite des attributs de cette classe. Synonymes RPPS : Diplôme obtenu</t>
+          <t>Un diplôme sanctionne un niveau de connaissances. L’Etat intervient, dans certains cas, sur le programme et la pédagogie de certains cursus diplômants, par exemple les diplômes d'Etat.La classe \"Diplome\" est une classe générale contenant les propriétés communes aux différents types de diplômes.Chaque diplôme est décrit dans le modèle comme une spécialisation de la classe Diplome et à ce titre, hérite des attributs de cette classe. Synonymes RPPS : Diplôme obtenu</t>
         </is>
       </c>
       <c r="G89" s="3" t="inlineStr"/>
@@ -8096,7 +8096,7 @@
       </c>
       <c r="F214" s="5" t="inlineStr">
         <is>
-          <t>Renseigné uniquement pour les certificats logiciels de portée Structure. Ce champ correspond au CN du DNSujet, il contient soit un "FQDN" pour les certificats de type serveur "SSL", soit un nom applicatif pour les autres certificats.</t>
+          <t>Renseigné uniquement pour les certificats logiciels de portée Structure. Ce champ correspond au CN du DNSujet, il contient soit un \"FQDN\" pour les certificats de type serveur \"SSL\", soit un nom applicatif pour les autres certificats.</t>
         </is>
       </c>
       <c r="G214" s="5" t="inlineStr"/>
@@ -8268,7 +8268,7 @@
       </c>
       <c r="F218" s="5" t="inlineStr">
         <is>
-          <t>Identification de l'émetteur du token complété du numéro de série de la carte.Cet attribut est renseigné obligatoirement pour les certificats embarqués dans les cartes CPS et optionnellement pour les modules de sécurité physique.Exemple : "8025000001/9999999999"  '8025000001' : Identifiant national de l'ANS'9999999999' : N° de série de la carte sur 10 chiffres</t>
+          <t>Identification de l'émetteur du token complété du numéro de série de la carte.Cet attribut est renseigné obligatoirement pour les certificats embarqués dans les cartes CPS et optionnellement pour les modules de sécurité physique.Exemple : \"8025000001/9999999999\"  '8025000001' : Identifiant national de l'ANS'9999999999' : N° de série de la carte sur 10 chiffres</t>
         </is>
       </c>
       <c r="G218" s="5" t="inlineStr"/>
@@ -8555,7 +8555,7 @@
       </c>
       <c r="F225" s="4" t="inlineStr">
         <is>
-          <t>Identifiant FINESS de l'entité juridique attribué lors de sa création.Les personnes morales identifiées par des numéros FINESS sont également dotées de numéros Siren.  Le numéro FINESS étant porteur intrinsèquement de liens avec le domaine sanitaire ou le domaine médico-social, il est, s'il existe, à privilégier pour l’identification de ces personnes morales en tant qu’acteurs sanitaires et médico-sociaux (Référentiel d’identification des acteurs sanitaires et médico-sociaux - Politique Générale de Sécurité des Systèmes d’Information de Santé (PGSSI-S)).Le numéro FINESS est composé de 9 caractères numériques, tels que:** Position 1-2 : numéro du département d'implantation ("2A", "2B" pour la Corse; "97" pour les départements d’Outre-mer; "98" pour Mayotte);** Position 3 : "0";** Position 4-8: "1" pour Guadeloupe, "2" pour Martinique, "3" pour Guyane, "4" pour Réunion, "5" pour Saint-Pierre-et-Miquelon + numéro d'ordre de 4 chiffres;** Position 4-8 : numéro d’ordre de 5 chiffres pour tous les autres départements;** Position 9 : clé de Luhn calculée automatiquement.</t>
+          <t>Identifiant FINESS de l'entité juridique attribué lors de sa création.Les personnes morales identifiées par des numéros FINESS sont également dotées de numéros Siren.  Le numéro FINESS étant porteur intrinsèquement de liens avec le domaine sanitaire ou le domaine médico-social, il est, s'il existe, à privilégier pour l’identification de ces personnes morales en tant qu’acteurs sanitaires et médico-sociaux (Référentiel d’identification des acteurs sanitaires et médico-sociaux - Politique Générale de Sécurité des Systèmes d’Information de Santé (PGSSI-S)).Le numéro FINESS est composé de 9 caractères numériques, tels que:** Position 1-2 : numéro du département d'implantation (\"2A\", \"2B\" pour la Corse; \"97\" pour les départements d’Outre-mer; \"98\" pour Mayotte);** Position 3 : \"0\";** Position 4-8: \"1\" pour Guadeloupe, \"2\" pour Martinique, \"3\" pour Guyane, \"4\" pour Réunion, \"5\" pour Saint-Pierre-et-Miquelon + numéro d'ordre de 4 chiffres;** Position 4-8 : numéro d’ordre de 5 chiffres pour tous les autres départements;** Position 9 : clé de Luhn calculée automatiquement.</t>
         </is>
       </c>
       <c r="G225" s="4" t="inlineStr"/>
@@ -9014,7 +9014,7 @@
       </c>
       <c r="F236" s="5" t="inlineStr">
         <is>
-          <t>Agrégat de statut juridique de niveau 1. L'agrégat de niveau 1 représente des regroupements d'agrégats de niveau 2. Par exemple, le code 1000 "Organismes et Etablissements publics" regroupe les codes d'agrégat de niveau 2 1100 et 1200.</t>
+          <t>Agrégat de statut juridique de niveau 1. L'agrégat de niveau 1 représente des regroupements d'agrégats de niveau 2. Par exemple, le code 1000 \"Organismes et Etablissements publics\" regroupe les codes d'agrégat de niveau 2 1100 et 1200.</t>
         </is>
       </c>
       <c r="G236" s="5" t="inlineStr">
@@ -9059,7 +9059,7 @@
       </c>
       <c r="F237" s="4" t="inlineStr">
         <is>
-          <t>Agrégat de statut juridique de niveau 2. L'agrégat de niveau 2 représente des regroupements d'agrégats de niveau 3. Par exemple, le code 1100 "Etat et Collectivités territoriales" regroupe les codes d'agrégats de niveau 3 1110 et 1120. Il caractérise le statut juridique d’une structure au sens du droit applicable (public / privé) et de la finalité (non lucratif / commercial).</t>
+          <t>Agrégat de statut juridique de niveau 2. L'agrégat de niveau 2 représente des regroupements d'agrégats de niveau 3. Par exemple, le code 1100 \"Etat et Collectivités territoriales\" regroupe les codes d'agrégats de niveau 3 1110 et 1120. Il caractérise le statut juridique d’une structure au sens du droit applicable (public / privé) et de la finalité (non lucratif / commercial).</t>
         </is>
       </c>
       <c r="G237" s="4" t="inlineStr">
@@ -9104,7 +9104,7 @@
       </c>
       <c r="F238" s="5" t="inlineStr">
         <is>
-          <t>Agrégat de statut juridique de niveau 3. L'agrégat de niveau 3 représente des regroupements de statuts juridiques. Par exemple, le code 1120 "Collectivité territoriale" regroupe les statuts juridiques 02, 03 etc.</t>
+          <t>Agrégat de statut juridique de niveau 3. L'agrégat de niveau 3 représente des regroupements de statuts juridiques. Par exemple, le code 1120 \"Collectivité territoriale\" regroupe les statuts juridiques 02, 03 etc.</t>
         </is>
       </c>
       <c r="G238" s="5" t="inlineStr">
@@ -9690,7 +9690,7 @@
       </c>
       <c r="F252" s="5" t="inlineStr">
         <is>
-          <t>Numéro FINESS de l'entité géographique.Le numéro FINESS étant porteur intrinsèquement de liens avec le domaine sanitaire ou le domaine médico-social, il est, s'il existe, à privilégier pour l’identification des entités géographiques en tant qu’acteurs sanitaires et médico-sociaux par rapport au numéro SIRET (Référentiel d’identification des acteurs sanitaires et médico-sociaux - Politique Générale de Sécurité des Systèmes d’Information de Santé (PGSSI-S)).A chaque EG (établissement) est attribué un numéro FINESS qui est composé de 9 caractères numériques, tels que :** Position 1-2 : numéro du département d'implantation ("2A", "2B" pour la Corse; "97" pour les départements d’Outre-mer; "98" pour Mayotte);** Position 3 : "0";** Position 4-8: "1" pour Guadeloupe, "2" pour Martinique, "3" pour Guyane, "4" pour Réunion, "5" pour Saint-Pierre-et-Miquelon + numéro d'ordre de 4 chiffres;** Position 4-8 : numéro d’ordre de 5 chiffres pour tous les autres départements;** Position 9 : clé de Luhn calculée automatiquement.</t>
+          <t>Numéro FINESS de l'entité géographique.Le numéro FINESS étant porteur intrinsèquement de liens avec le domaine sanitaire ou le domaine médico-social, il est, s'il existe, à privilégier pour l’identification des entités géographiques en tant qu’acteurs sanitaires et médico-sociaux par rapport au numéro SIRET (Référentiel d’identification des acteurs sanitaires et médico-sociaux - Politique Générale de Sécurité des Systèmes d’Information de Santé (PGSSI-S)).A chaque EG (établissement) est attribué un numéro FINESS qui est composé de 9 caractères numériques, tels que :** Position 1-2 : numéro du département d'implantation (\"2A\", \"2B\" pour la Corse; \"97\" pour les départements d’Outre-mer; \"98\" pour Mayotte);** Position 3 : \"0\";** Position 4-8: \"1\" pour Guadeloupe, \"2\" pour Martinique, \"3\" pour Guyane, \"4\" pour Réunion, \"5\" pour Saint-Pierre-et-Miquelon + numéro d'ordre de 4 chiffres;** Position 4-8 : numéro d’ordre de 5 chiffres pour tous les autres départements;** Position 9 : clé de Luhn calculée automatiquement.</t>
         </is>
       </c>
       <c r="G252" s="5" t="inlineStr"/>
@@ -9899,7 +9899,7 @@
       </c>
       <c r="F257" s="4" t="inlineStr">
         <is>
-          <t>Le "numéro éducation nationale de l'établissement" est un numéro associé délivré par l’Éducation nationale, pour tous les établissements et services pour enfants et adolescents handicapés qui emploient du personnel de l’Education nationale.</t>
+          <t>Le \"numéro éducation nationale de l'établissement\" est un numéro associé délivré par l’Éducation nationale, pour tous les établissements et services pour enfants et adolescents handicapés qui emploient du personnel de l’Education nationale.</t>
         </is>
       </c>
       <c r="G257" s="4" t="inlineStr"/>
@@ -9981,7 +9981,7 @@
       </c>
       <c r="F259" s="4" t="inlineStr">
         <is>
-          <t>Nom sous lequel l'entité géographique exerce son activité. Il s’agit, par exemple, de l’enseigne commerciale pour les pharmacies. Dans le cas d'un établissement enregistré dans le FINESS, cet attribut correspond à la notion de "raison sociale d'un établissement" renseignée dans le FINESS.</t>
+          <t>Nom sous lequel l'entité géographique exerce son activité. Il s’agit, par exemple, de l’enseigne commerciale pour les pharmacies. Dans le cas d'un établissement enregistré dans le FINESS, cet attribut correspond à la notion de \"raison sociale d'un établissement\" renseignée dans le FINESS.</t>
         </is>
       </c>
       <c r="G259" s="4" t="inlineStr"/>
@@ -10321,7 +10321,7 @@
       </c>
       <c r="F267" s="4" t="inlineStr">
         <is>
-          <t>Agrégat de catégories d'établissements de niveau 1. L'agrégat de niveau 1 représente des regroupements d'agrégat de niveau 2. Par exemple, le code 1000 "Etablissement relevant de la loi hospitalière" regroupe les codes d'agrégat de niveau 2 1100 et 1200.</t>
+          <t>Agrégat de catégories d'établissements de niveau 1. L'agrégat de niveau 1 représente des regroupements d'agrégat de niveau 2. Par exemple, le code 1000 \"Etablissement relevant de la loi hospitalière\" regroupe les codes d'agrégat de niveau 2 1100 et 1200.</t>
         </is>
       </c>
       <c r="G267" s="4" t="inlineStr">
@@ -10366,7 +10366,7 @@
       </c>
       <c r="F268" s="5" t="inlineStr">
         <is>
-          <t>Agrégat de catégories d'établissements de niveau 2. L'agrégat de niveau 2 représente des regroupements d'agrégats de niveau 3. Par exemple, le code 1100 "Etablissement hospitaliers" regroupe les codes d'agrégat de niveau 3 1101, 1102, etc.</t>
+          <t>Agrégat de catégories d'établissements de niveau 2. L'agrégat de niveau 2 représente des regroupements d'agrégats de niveau 3. Par exemple, le code 1100 \"Etablissement hospitaliers\" regroupe les codes d'agrégat de niveau 3 1101, 1102, etc.</t>
         </is>
       </c>
       <c r="G268" s="5" t="inlineStr">
@@ -10411,7 +10411,7 @@
       </c>
       <c r="F269" s="4" t="inlineStr">
         <is>
-          <t>Agrégat de catégories d'établissements de niveau 3. L'agrégat de niveau 3 représente des regroupements de catégories d'établissement. Par exemple, le code 1101 "Centres hospitaliers régionaux" regroupe les catégories d'établissement 101, 106 etc.</t>
+          <t>Agrégat de catégories d'établissements de niveau 3. L'agrégat de niveau 3 représente des regroupements de catégories d'établissement. Par exemple, le code 1101 \"Centres hospitaliers régionaux\" regroupe les catégories d'établissement 101, 106 etc.</t>
         </is>
       </c>
       <c r="G269" s="4" t="inlineStr">
@@ -10591,7 +10591,7 @@
       </c>
       <c r="F273" s="4" t="inlineStr">
         <is>
-          <t>Nature du budget alloué à l'établissement dont les valeurs sont "G" pour général et "A" pour annexe.</t>
+          <t>Nature du budget alloué à l'établissement dont les valeurs sont \"G\" pour général et \"A\" pour annexe.</t>
         </is>
       </c>
       <c r="G273" s="4" t="inlineStr"/>
@@ -12825,7 +12825,7 @@
       </c>
       <c r="F327" s="4" t="inlineStr">
         <is>
-          <t>Les modalités sont des modes d’application ou des types de soins prévus par les textes réglementaires encadrant chaque activité de soins. Ce sont des pratiques thérapeutiques. Une activité de soins peut ou non avoir des modalités (dans ce cas, le code de la modalité est "00"). Les modalités peuvent être communes à plusieurs activités de soins ou spécifiques à une seule.</t>
+          <t>Les modalités sont des modes d’application ou des types de soins prévus par les textes réglementaires encadrant chaque activité de soins. Ce sont des pratiques thérapeutiques. Une activité de soins peut ou non avoir des modalités (dans ce cas, le code de la modalité est \"00\"). Les modalités peuvent être communes à plusieurs activités de soins ou spécifiques à une seule.</t>
         </is>
       </c>
       <c r="G327" s="4" t="inlineStr">
@@ -13247,7 +13247,7 @@
       </c>
       <c r="F337" s="4" t="inlineStr">
         <is>
-          <t>Les modalités sont des modes d’application ou des types de soins prévus par les textes réglementaires encadrant chaque activité de soins. Ce sont des pratiques thérapeutiques. Une activité de soins peut ou non avoir des modalités (dans ce cas, le code de la modalité est "00"). Les modalités peuvent être communes à plusieurs activités de soins ou spécifiques à une seule.</t>
+          <t>Les modalités sont des modes d’application ou des types de soins prévus par les textes réglementaires encadrant chaque activité de soins. Ce sont des pratiques thérapeutiques. Une activité de soins peut ou non avoir des modalités (dans ce cas, le code de la modalité est \"00\"). Les modalités peuvent être communes à plusieurs activités de soins ou spécifiques à une seule.</t>
         </is>
       </c>
       <c r="G337" s="4" t="inlineStr">
@@ -13546,7 +13546,7 @@
       </c>
       <c r="F344" s="5" t="inlineStr">
         <is>
-          <t>Les modalités sont des modes d’application ou des types de soins prévus par les textes réglementaires encadrant chaque activité de soins. Ce sont des pratiques thérapeutiques. Une activité de soins peut ou non avoir des modalités (dans ce cas, le code de la modalité est "00"). Les modalités peuvent être communes à plusieurs activités de soins ou spécifiques à une seule.</t>
+          <t>Les modalités sont des modes d’application ou des types de soins prévus par les textes réglementaires encadrant chaque activité de soins. Ce sont des pratiques thérapeutiques. Une activité de soins peut ou non avoir des modalités (dans ce cas, le code de la modalité est \"00\"). Les modalités peuvent être communes à plusieurs activités de soins ou spécifiques à une seule.</t>
         </is>
       </c>
       <c r="G344" s="5" t="inlineStr">
@@ -15914,7 +15914,7 @@
       </c>
       <c r="F400" s="5" t="inlineStr">
         <is>
-          <t>Identifiant de l'offre, unique et persistant au niveau national, généré par une instance régionale du ROR ou par le ROR national.Format : Concaténation du code INSEE région et d’un identifiant généré, par le ROR régional ou le ROR national, séparé par le caractère "slash" (ex: 94/666).</t>
+          <t>Identifiant de l'offre, unique et persistant au niveau national, généré par une instance régionale du ROR ou par le ROR national.Format : Concaténation du code INSEE région et d’un identifiant généré, par le ROR régional ou le ROR national, séparé par le caractère \"slash\" (ex: 94/666).</t>
         </is>
       </c>
       <c r="G400" s="5" t="inlineStr"/>
@@ -18917,7 +18917,7 @@
       </c>
       <c r="F471" s="4" t="inlineStr">
         <is>
-          <t>Titre de la convention, par exemple "Convention constitutive du groupement hospitalier de territoire des Bouches du Rhône".</t>
+          <t>Titre de la convention, par exemple \"Convention constitutive du groupement hospitalier de territoire des Bouches du Rhône\".</t>
         </is>
       </c>
       <c r="G471" s="4" t="inlineStr"/>
@@ -19573,7 +19573,7 @@
       </c>
       <c r="F487" s="4" t="inlineStr">
         <is>
-          <t>Le nom de  naissance est un élément d’identité mentionné à l’article R. 1111-8-6 du CSP.C'est  un trait "strict" d'identité de la personne dans l'INS ( Référentiel Identité Nationale de Santé)synonyme moins précis : nom de famille</t>
+          <t>Le nom de  naissance est un élément d’identité mentionné à l’article R. 1111-8-6 du CSP.C'est  un trait \"strict\" d'identité de la personne dans l'INS ( Référentiel Identité Nationale de Santé)synonyme moins précis : nom de famille</t>
         </is>
       </c>
       <c r="G487" s="4" t="inlineStr"/>
@@ -19614,7 +19614,7 @@
       </c>
       <c r="F488" s="5" t="inlineStr">
         <is>
-          <t>Liste des prénoms de naissance indiqués sur l'acte de naissance. Ce sont des éléments d’identité mentionnés à l’article R. 1111-8-6 du CSP.La liste des prénoms de naissance est un trait d'identité "strict" de la personne dans l'INS ( Référentiel Identité Nationale de Santé)  Ce champ peut comporter plusieurs prénoms, simples ou composés.(avec ou sans tiret d’union entre les prénoms).</t>
+          <t>Liste des prénoms de naissance indiqués sur l'acte de naissance. Ce sont des éléments d’identité mentionnés à l’article R. 1111-8-6 du CSP.La liste des prénoms de naissance est un trait d'identité \"strict\" de la personne dans l'INS ( Référentiel Identité Nationale de Santé)  Ce champ peut comporter plusieurs prénoms, simples ou composés.(avec ou sans tiret d’union entre les prénoms).</t>
         </is>
       </c>
       <c r="G488" s="5" t="inlineStr"/>
@@ -25181,7 +25181,7 @@
       </c>
       <c r="F623" s="4" t="inlineStr">
         <is>
-          <t>Statut du créneau. Il est fixé à "libre".</t>
+          <t>Statut du créneau. Il est fixé à \"libre\".</t>
         </is>
       </c>
       <c r="G623" s="4" t="inlineStr"/>
@@ -26329,7 +26329,7 @@
       </c>
       <c r="F651" s="4" t="inlineStr">
         <is>
-          <t>Statut de la plage de disponibilité : Par défaut le statut est à "disponible". Par exception, il est possible de déclarer une indisponibilité. Le statut est alors à "indisponible".</t>
+          <t>Statut de la plage de disponibilité : Par défaut le statut est à \"disponible\". Par exception, il est possible de déclarer une indisponibilité. Le statut est alors à \"indisponible\".</t>
         </is>
       </c>
       <c r="G651" s="4" t="inlineStr"/>
@@ -26944,7 +26944,7 @@
       </c>
       <c r="F666" s="5" t="inlineStr">
         <is>
-          <t>Indicateur pour specifier si le dispositif est actif. L’article 2 partie 4 du Règlement (UE) 2017/745 du 5 avril 2017 définit les dispositifs actifs comme "tout dispositif dont le fonctionnement dépend d'une source d'énergie autre que celle générée par le corps humain à cette fin ou par la pesanteur et agissant par modification de la densité de cette énergie ou par conversion de celle-ci. Les dispositifs destinés à la transmission d'énergie, de substances ou d'autres éléments, sans modification significative, entre un dispositif actif et le patient ne sont pas réputés être des dispositifs actifs. Les logiciels sont aussi réputés être des dispositifs actifs." 1 : dispositif actif0 : dispositif non actif</t>
+          <t>Indicateur pour specifier si le dispositif est actif. L’article 2 partie 4 du Règlement (UE) 2017/745 du 5 avril 2017 définit les dispositifs actifs comme \"tout dispositif dont le fonctionnement dépend d'une source d'énergie autre que celle générée par le corps humain à cette fin ou par la pesanteur et agissant par modification de la densité de cette énergie ou par conversion de celle-ci. Les dispositifs destinés à la transmission d'énergie, de substances ou d'autres éléments, sans modification significative, entre un dispositif actif et le patient ne sont pas réputés être des dispositifs actifs. Les logiciels sont aussi réputés être des dispositifs actifs.\" 1 : dispositif actif0 : dispositif non actif</t>
         </is>
       </c>
       <c r="G666" s="5" t="inlineStr"/>
@@ -29579,7 +29579,7 @@
       </c>
       <c r="F729" s="4" t="inlineStr">
         <is>
-          <t>Situation familiale de la personne (célibataire, divorcée, etc.).Les valeurs de ce code sont répertoriées dans plusieurs nomenclatures notamment:- la liste de la Déclaration Automatisée des Données Sociales Unifiée (DADS-U):01: célibataire02: marié(e)03: divorcé(e)04: séparé(e)05: veuf, veuve06: vie maritale07: PACS90: non connueetc.- Liste de codes HL7 "MaritalStatus":A: Annulled, marriage contract has been declared null and to not have existedD: Divorced, marriage contract has been declared dissolved and inactiveI: Interlocutory, subject to an Interlocutory DecreeL: Legally separatedM: Married, a current marriage contract is activeP: Polygamous, more than 1 current spouseS: Never Married, no marriage contract has ever been enteredT: Domestic partner, person declares that a domestic partner relationship exists.U: Unmarried, currently not in a marriage contract.W: Widowed, the spouse has died</t>
+          <t>Situation familiale de la personne (célibataire, divorcée, etc.).Les valeurs de ce code sont répertoriées dans plusieurs nomenclatures notamment:- la liste de la Déclaration Automatisée des Données Sociales Unifiée (DADS-U):01: célibataire02: marié(e)03: divorcé(e)04: séparé(e)05: veuf, veuve06: vie maritale07: PACS90: non connueetc.- Liste de codes HL7 \"MaritalStatus\":A: Annulled, marriage contract has been declared null and to not have existedD: Divorced, marriage contract has been declared dissolved and inactiveI: Interlocutory, subject to an Interlocutory DecreeL: Legally separatedM: Married, a current marriage contract is activeP: Polygamous, more than 1 current spouseS: Never Married, no marriage contract has ever been enteredT: Domestic partner, person declares that a domestic partner relationship exists.U: Unmarried, currently not in a marriage contract.W: Widowed, the spouse has died</t>
         </is>
       </c>
       <c r="G729" s="4" t="inlineStr"/>
@@ -31976,7 +31976,7 @@
       </c>
       <c r="F786" s="5" t="inlineStr">
         <is>
-          <t>Texte libre donnant les coordonnées de la (ou des) personne(s) responsable(s) au niveau opérationnel de la boîte aux lettres. Non renseigné pour les types de boîte aux lettres "PER".</t>
+          <t>Texte libre donnant les coordonnées de la (ou des) personne(s) responsable(s) au niveau opérationnel de la boîte aux lettres. Non renseigné pour les types de boîte aux lettres \"PER\".</t>
         </is>
       </c>
       <c r="G786" s="5" t="inlineStr"/>
@@ -32849,7 +32849,7 @@
       </c>
       <c r="F807" s="4" t="inlineStr">
         <is>
-          <t>Code officiel géographique (COG), diffusé par l'INSEE, de la commune d'implantation du destinataire. Ce code ne fait pas partie de la norme NF Z 10-011 mais il correspond au libellé de l'attribut "localite" de la classe Adresse qui lui fait partie de la norme.</t>
+          <t>Code officiel géographique (COG), diffusé par l'INSEE, de la commune d'implantation du destinataire. Ce code ne fait pas partie de la norme NF Z 10-011 mais il correspond au libellé de l'attribut \"localite\" de la classe Adresse qui lui fait partie de la norme.</t>
         </is>
       </c>
       <c r="G807" s="4" t="inlineStr">
@@ -32976,7 +32976,7 @@
       </c>
       <c r="F810" s="5" t="inlineStr">
         <is>
-          <t>Indique le ou les types d'adresse tel que "Adresse du domicile", "Adresse professionnelle", "Adresse de facturation", "Adresse postale", "Adresse géographique", etc.Cet attribut ne fait pas partie de la norme  NF Z 10-011.</t>
+          <t>Indique le ou les types d'adresse tel que \"Adresse du domicile\", \"Adresse professionnelle\", \"Adresse de facturation\", \"Adresse postale\", \"Adresse géographique\", etc.Cet attribut ne fait pas partie de la norme  NF Z 10-011.</t>
         </is>
       </c>
       <c r="G810" s="5" t="inlineStr"/>
@@ -34107,7 +34107,7 @@
       </c>
       <c r="F837" s="4" t="inlineStr">
         <is>
-          <t>Une mesure de la distance angulaire nord ou sud depuis l'équateur jusqu'au parallèle du spécifique.L'unité de mesure est spécifiée dans le type "Mesure". Le choix est possible entre le Degré Décimal (DD) et le Degré Minute Seconde (DMS), l'unité de mesure est obligatoire dans l'échange.</t>
+          <t>Une mesure de la distance angulaire nord ou sud depuis l'équateur jusqu'au parallèle du spécifique.L'unité de mesure est spécifiée dans le type \"Mesure\". Le choix est possible entre le Degré Décimal (DD) et le Degré Minute Seconde (DMS), l'unité de mesure est obligatoire dans l'échange.</t>
         </is>
       </c>
       <c r="G837" s="4" t="inlineStr"/>
@@ -34193,7 +34193,7 @@
       </c>
       <c r="F839" s="4" t="inlineStr">
         <is>
-          <t>Une mesure de la distance angulaire est ou ouest depuis le méridien de Greenwich jusqu'au méridien du point spécifiqueL'unité de mesure est spécifiée dans le type "Mesure". Le choix est possible entre le Degré Décimal (DD) et le Degré Minute Seconde (DMS), l'unité de mesure est obligatoire dans l'échange.</t>
+          <t>Une mesure de la distance angulaire est ou ouest depuis le méridien de Greenwich jusqu'au méridien du point spécifiqueL'unité de mesure est spécifiée dans le type \"Mesure\". Le choix est possible entre le Degré Décimal (DD) et le Degré Minute Seconde (DMS), l'unité de mesure est obligatoire dans l'échange.</t>
         </is>
       </c>
       <c r="G839" s="4" t="inlineStr"/>
@@ -34320,7 +34320,7 @@
       </c>
       <c r="F842" s="5" t="inlineStr">
         <is>
-          <t>Une mesure de la hauteur du point spécifique par rapport au niveau de la mer. L'unité de mesure est spécifiée dans le type "Mesure". En général, l'unité de mesure choisie est le mètre.</t>
+          <t>Une mesure de la hauteur du point spécifique par rapport au niveau de la mer. L'unité de mesure est spécifiée dans le type \"Mesure\". En général, l'unité de mesure choisie est le mètre.</t>
         </is>
       </c>
       <c r="G842" s="5" t="inlineStr"/>

</xml_diff>